<commit_message>
fix: align Forge vent arrivals and prove active reduced motion
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V158.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V158.xlsx
@@ -2168,12 +2168,12 @@
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">b48b0a0762e7df1c2ef9c6aa8af4a412c42584936768467ae8dc60889ed16928</t>
+          <t xml:space="preserve">5bbc1fd5546e55c7f82c13d5f1b2962e8f49a00c5baf5c614b2a9ade81d14491</t>
         </is>
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les PNJ Forge bornés gardent leur identité éditable, leur récit et les admissions natives dans les deux playtests, copies et échanges de documents.</t>
+          <t xml:space="preserve">Les volumes de conduits gardent le refus des corps PNJ ; les arrivées Mission conservent leurs conduits non bloquants et les arrivées Vaisseau leurs obstacles natifs.</t>
         </is>
       </c>
       <c r="E24" s="0" t="inlineStr">
@@ -19366,7 +19366,7 @@
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">16 PNJ/salle ; 64 PNJ/projet ; nom 80 caractères ; apparences coloniales existantes.</t>
+          <t xml:space="preserve">16 PNJ/salle ; 64 PNJ/projet ; nom 80 caractères ; conduits refusés pour les corps PNJ, arrivées Mission non bloquées par ces conduits.</t>
         </is>
       </c>
       <c r="D17" s="0" t="inlineStr">
@@ -19966,7 +19966,7 @@
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trois plaques natives, contacts et raccord sans écriture physique.</t>
+          <t xml:space="preserve">Trois plaques natives, contacts et raccord sans écriture physique ; preuve navigateur du mouvement réduit au même tick natif, avant 43 ticks de prise.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: prewarm selected modular outfits within active texture budget
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V158.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V158.xlsx
@@ -111,8 +111,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV158Table11" displayName="AuditV158Table11" ref="A5:E32" totalsRowShown="0">
-  <autoFilter ref="A5:E32"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV158Table11" displayName="AuditV158Table11" ref="A5:E33" totalsRowShown="0">
+  <autoFilter ref="A5:E33"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Module"/>
     <tableColumn id="2" name="SHA V157"/>
@@ -181,8 +181,8 @@
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="AuditV158Table15" displayName="AuditV158Table15" ref="A5:G9" totalsRowShown="0">
-  <autoFilter ref="A5:G9"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="AuditV158Table15" displayName="AuditV158Table15" ref="A5:G10" totalsRowShown="0">
+  <autoFilter ref="A5:G10"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Lot_ID"/>
     <tableColumn id="2" name="Contrat"/>
@@ -262,8 +262,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="AuditV158Table6" displayName="AuditV158Table6" ref="A5:E19" totalsRowShown="0">
-  <autoFilter ref="A5:E19"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="AuditV158Table6" displayName="AuditV158Table6" ref="A5:E20" totalsRowShown="0">
+  <autoFilter ref="A5:E20"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Source_ID"/>
     <tableColumn id="2" name="Type"/>
@@ -532,8 +532,8 @@
         </is>
       </c>
       <c r="E22" s="0">
-        <f>COUNTA('15_LotsV158'!A6:A9)</f>
-        <v>4</v>
+        <f>COUNTA('15_LotsV158'!A6:A10)</f>
+        <v>5</v>
       </c>
     </row>
     <row r="23" ht="48" customHeight="1">
@@ -2347,7 +2347,7 @@
     <row r="31" ht="48" customHeight="1">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/save.js</t>
+          <t xml:space="preserve">src/player-appearance-runtime-v126.js</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
@@ -2357,42 +2357,69 @@
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">43391c19bb2617d7e9afaa17de2a79616af3fe510f24453cdd9e45b43ebc1678</t>
+          <t xml:space="preserve">6216b2066114e30b628807ab2eef1ff1ed742ce277aa216a3cef8927b337b78a</t>
         </is>
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les nouveaux états de présentation et de circulation sont normalisés sans inventer de trajet accompli ni rejouer une ancienne libération.</t>
+          <t xml:space="preserve">Les textures courantes des opérateurs et leurs équipements restent prioritaires ; le kit sélectionné et les futures bases sont préparés dans le budget natif de seize images, sans attendre le décodage.</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-npc-circulation-v158.mjs ; scripts/verify-black-cocoon-presentation-v158.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-appearance-runtime-v126.mjs</t>
         </is>
       </c>
     </row>
     <row r="32" ht="48" customHeight="1">
       <c r="A32" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">src/save.js</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non épinglé en V157</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">43391c19bb2617d7e9afaa17de2a79616af3fe510f24453cdd9e45b43ebc1678</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les nouveaux états de présentation et de circulation sont normalisés sans inventer de trajet accompli ni rejouer une ancienne libération.</t>
+        </is>
+      </c>
+      <c r="E32" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-npc-circulation-v158.mjs ; scripts/verify-black-cocoon-presentation-v158.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="48" customHeight="1">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">src/xeno-trials-capture-reception-v158.js</t>
         </is>
       </c>
-      <c r="B32" s="0" t="inlineStr">
+      <c r="B33" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Non épinglé en V157</t>
         </is>
       </c>
-      <c r="C32" s="0" t="inlineStr">
+      <c r="C33" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">223b5b41fb00091f78b596866985108e4bced494fa41ad1c81b1054c064fb314</t>
         </is>
       </c>
-      <c r="D32" s="0" t="inlineStr">
+      <c r="D33" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Trois réceptions de simulation utilisent leurs plaques natives exactes et rejoignent la prise existante sans modifier corps physiques ni verdict.</t>
         </is>
       </c>
-      <c r="E32" s="0" t="inlineStr">
+      <c r="E33" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">scripts/verify-xeno-trials-capture-reception-v158.mjs ; scripts/verify-xeno-trials-rig-v154.mjs</t>
         </is>
@@ -13701,6 +13728,43 @@
         </is>
       </c>
     </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">modular-costume-readiness</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Préparation des costumes modulaires</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Opérateurs et kit colonial sélectionné ; budget natif de seize images</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implémenté (préparation bornée)</t>
+        </is>
+      </c>
+      <c r="E10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">À exécuter sur le commit publié</t>
+        </is>
+      </c>
+      <c r="F10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Images natives déjà livrées ; aucun nouveau pixel ni canon</t>
+        </is>
+      </c>
+      <c r="G10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30 costumes franchise sans atlas dédié ; disponibilité et pression du cache restent des limites.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -19823,6 +19887,33 @@
         </is>
       </c>
     </row>
+    <row r="20" ht="48" customHeight="1">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRC-COSTUME-READINESS-V158</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contrat exécutable</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/player-appearance-runtime-v126.js</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Textures courantes prioritaires ; préparation du kit et de futures bases dans le budget natif de seize images.</t>
+        </is>
+      </c>
+      <c r="E20" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dépend de la disponibilité des images ; pas de nouvel atlas franchise ni de garantie sous pression maximale du cache.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -20032,7 +20123,7 @@
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Captures et contrôles mesurés seulement après recette, sans participants humains inventés.</t>
+          <t xml:space="preserve">Captures et contrôles mesurés après recette ; préparation du kit vérifiée après disponibilité initiale des images, sans participants humains inventés.</t>
         </is>
       </c>
     </row>

</xml_diff>